<commit_message>
Refactor and flatten CMETS extractor pipeline
</commit_message>
<xml_diff>
--- a/Connectivity Application Data.xlsx
+++ b/Connectivity Application Data.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\CTU-automated-pdf-extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93662958-8F8F-4955-B491-D508AF8F2483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E14165F-19D5-4C36-9A08-5F886AD5D019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Sources" sheetId="1" r:id="rId1"/>
     <sheet name="Data to be captured" sheetId="2" r:id="rId2"/>
-    <sheet name="RE Potential" sheetId="3" r:id="rId3"/>
-    <sheet name="Margin" sheetId="4" r:id="rId4"/>
-    <sheet name="Non RE proposed RE Integration" sheetId="5" r:id="rId5"/>
-    <sheet name="Transformation Capacity" sheetId="6" r:id="rId6"/>
-    <sheet name="Element Status" sheetId="7" r:id="rId7"/>
+    <sheet name="Bulk Consumers" sheetId="8" r:id="rId3"/>
+    <sheet name="RE Potential" sheetId="3" r:id="rId4"/>
+    <sheet name="Margin" sheetId="4" r:id="rId5"/>
+    <sheet name="Non RE proposed RE Integration" sheetId="5" r:id="rId6"/>
+    <sheet name="Transformation Capacity" sheetId="6" r:id="rId7"/>
+    <sheet name="Element Status" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="226">
   <si>
     <t>SN</t>
   </si>
@@ -687,13 +688,46 @@
   </si>
   <si>
     <t>CMETS</t>
+  </si>
+  <si>
+    <t>Connectivity Under Process</t>
+  </si>
+  <si>
+    <t>Hydro</t>
+  </si>
+  <si>
+    <t>GNA Application ID</t>
+  </si>
+  <si>
+    <t>GNA Type</t>
+  </si>
+  <si>
+    <t>Quantum (MW)</t>
+  </si>
+  <si>
+    <t>Within Region</t>
+  </si>
+  <si>
+    <t>Outside Region</t>
+  </si>
+  <si>
+    <t>Total Quantum (MW)</t>
+  </si>
+  <si>
+    <t>Status of application (Applied/Withdrawn / Granted. Revoked.)</t>
+  </si>
+  <si>
+    <t>Start Date of GNA</t>
+  </si>
+  <si>
+    <t>End Date of GNA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -760,8 +794,27 @@
       <sz val="10"/>
       <name val="Adani Regular"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Adani Regular"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Adani Regular"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Adani Regular"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -792,8 +845,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCAEDFB"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -953,13 +1012,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1069,6 +1148,34 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="distributed" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="distributed" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1655,7 +1762,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AU9"/>
+  <dimension ref="A1:AV9"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="41.26953125" customWidth="1"/>
@@ -1668,24 +1775,24 @@
     <col min="16" max="16" width="13.54296875" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
     <col min="18" max="18" width="10.54296875" customWidth="1"/>
-    <col min="30" max="30" width="15.7265625" customWidth="1"/>
-    <col min="31" max="31" width="11.36328125" customWidth="1"/>
-    <col min="32" max="32" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="16" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="23.26953125" bestFit="1" customWidth="1"/>
-    <col min="36" max="37" width="16" customWidth="1"/>
-    <col min="38" max="38" width="8" customWidth="1"/>
-    <col min="39" max="39" width="10.453125" customWidth="1"/>
-    <col min="40" max="40" width="13.54296875" customWidth="1"/>
-    <col min="41" max="41" width="13.7265625" customWidth="1"/>
-    <col min="42" max="43" width="11.54296875" customWidth="1"/>
-    <col min="44" max="44" width="10.81640625" hidden="1" customWidth="1"/>
-    <col min="45" max="45" width="13" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="18.1796875" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="15.7265625" customWidth="1"/>
+    <col min="32" max="32" width="11.36328125" customWidth="1"/>
+    <col min="33" max="33" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="16" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="16" customWidth="1"/>
+    <col min="39" max="39" width="8" customWidth="1"/>
+    <col min="40" max="40" width="10.453125" customWidth="1"/>
+    <col min="41" max="41" width="13.54296875" customWidth="1"/>
+    <col min="42" max="42" width="13.7265625" customWidth="1"/>
+    <col min="43" max="44" width="11.54296875" customWidth="1"/>
+    <col min="45" max="45" width="10.81640625" hidden="1" customWidth="1"/>
+    <col min="46" max="46" width="13" hidden="1" customWidth="1"/>
+    <col min="47" max="47" width="18.1796875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="50">
+    <row r="1" spans="1:48" ht="50">
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
@@ -1723,44 +1830,45 @@
       <c r="T1" s="14"/>
       <c r="U1" s="14"/>
       <c r="V1" s="14"/>
-      <c r="W1" s="14">
+      <c r="W1" s="14"/>
+      <c r="X1" s="14">
         <v>300</v>
       </c>
-      <c r="X1" s="14"/>
       <c r="Y1" s="14"/>
       <c r="Z1" s="14"/>
       <c r="AA1" s="14"/>
-      <c r="AB1" s="14" t="s">
-        <v>208</v>
-      </c>
+      <c r="AB1" s="14"/>
       <c r="AC1" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="AD1" s="14"/>
+      <c r="AD1" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="AE1" s="14"/>
       <c r="AF1" s="14"/>
       <c r="AG1" s="14"/>
       <c r="AH1" s="14"/>
       <c r="AI1" s="14"/>
-      <c r="AJ1" s="26" t="s">
+      <c r="AJ1" s="14"/>
+      <c r="AK1" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="AK1" s="14" t="s">
+      <c r="AL1" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="AL1" s="14" t="s">
+      <c r="AM1" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="AM1" s="14"/>
       <c r="AN1" s="14"/>
       <c r="AO1" s="14"/>
       <c r="AP1" s="14"/>
       <c r="AQ1" s="14"/>
       <c r="AR1" s="14"/>
       <c r="AS1" s="14"/>
-      <c r="AU1" s="14"/>
-    </row>
-    <row r="2" spans="1:47" ht="89.25" customHeight="1">
+      <c r="AT1" s="14"/>
+      <c r="AV1" s="14"/>
+    </row>
+    <row r="2" spans="1:48" ht="89.25" customHeight="1">
       <c r="B2" s="7" t="s">
         <v>29</v>
       </c>
@@ -1817,76 +1925,77 @@
       </c>
       <c r="T2" s="4"/>
       <c r="U2" s="4"/>
-      <c r="V2" s="18" t="s">
+      <c r="V2" s="42"/>
+      <c r="W2" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="W2" s="19"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="18" t="s">
+      <c r="X2" s="19"/>
+      <c r="Y2" s="20"/>
+      <c r="Z2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="Z2" s="19"/>
       <c r="AA2" s="19"/>
-      <c r="AB2" s="3" t="s">
+      <c r="AB2" s="19"/>
+      <c r="AC2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="AC2" s="3"/>
-      <c r="AD2" s="1" t="s">
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AG2" s="5" t="s">
+      <c r="AH2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AH2" s="5" t="s">
+      <c r="AI2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="AI2" s="5" t="s">
+      <c r="AJ2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AJ2" s="5" t="s">
+      <c r="AK2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AK2" s="37" t="s">
+      <c r="AL2" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="AL2" s="10" t="s">
+      <c r="AM2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="AM2" s="1" t="s">
+      <c r="AN2" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="AN2" s="1" t="s">
+      <c r="AO2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AO2" s="1" t="s">
+      <c r="AP2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="AP2" s="1" t="s">
+      <c r="AQ2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AQ2" s="1" t="s">
+      <c r="AR2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AS2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AS2" s="1" t="s">
+      <c r="AT2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="AU2" s="1" t="s">
+      <c r="AV2" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:47" ht="31" customHeight="1">
+    <row r="3" spans="1:48" ht="31" customHeight="1">
       <c r="B3" s="8"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1914,36 +2023,38 @@
         <v>70</v>
       </c>
       <c r="V3" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="W3" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="X3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="Y3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="Z3" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="Z3" s="6" t="s">
+      <c r="AA3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="AA3" s="6" t="s">
+      <c r="AB3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="AB3" s="2" t="s">
+      <c r="AC3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AC3" s="2" t="s">
+      <c r="AD3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
-      <c r="AI3" s="9"/>
-      <c r="AJ3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="9"/>
       <c r="AK3" s="2"/>
       <c r="AL3" s="2"/>
       <c r="AM3" s="2"/>
@@ -1951,11 +2062,12 @@
       <c r="AO3" s="2"/>
       <c r="AP3" s="2"/>
       <c r="AQ3" s="2"/>
-      <c r="AR3" s="17"/>
-      <c r="AS3" s="2"/>
-      <c r="AU3" s="2"/>
-    </row>
-    <row r="5" spans="1:47">
+      <c r="AR3" s="2"/>
+      <c r="AS3" s="17"/>
+      <c r="AT3" s="2"/>
+      <c r="AV3" s="2"/>
+    </row>
+    <row r="5" spans="1:48">
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -1983,9 +2095,7 @@
       <c r="Z5" s="14"/>
       <c r="AA5" s="14"/>
       <c r="AB5" s="14"/>
-      <c r="AC5" s="14">
-        <v>996</v>
-      </c>
+      <c r="AC5" s="14"/>
       <c r="AD5" s="14"/>
       <c r="AE5" s="14"/>
       <c r="AF5" s="14"/>
@@ -2002,9 +2112,10 @@
       <c r="AQ5" s="14"/>
       <c r="AR5" s="14"/>
       <c r="AS5" s="14"/>
-      <c r="AU5" s="14"/>
-    </row>
-    <row r="6" spans="1:47">
+      <c r="AT5" s="14"/>
+      <c r="AV5" s="14"/>
+    </row>
+    <row r="6" spans="1:48">
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
       <c r="D6" s="14"/>
@@ -2049,9 +2160,10 @@
       <c r="AQ6" s="14"/>
       <c r="AR6" s="14"/>
       <c r="AS6" s="14"/>
-      <c r="AU6" s="14"/>
-    </row>
-    <row r="7" spans="1:47">
+      <c r="AT6" s="14"/>
+      <c r="AV6" s="14"/>
+    </row>
+    <row r="7" spans="1:48">
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -2096,9 +2208,10 @@
       <c r="AQ7" s="14"/>
       <c r="AR7" s="14"/>
       <c r="AS7" s="14"/>
-      <c r="AU7" s="14"/>
-    </row>
-    <row r="9" spans="1:47">
+      <c r="AT7" s="14"/>
+      <c r="AV7" s="14"/>
+    </row>
+    <row r="9" spans="1:48">
       <c r="A9" t="s">
         <v>76</v>
       </c>
@@ -2110,6 +2223,112 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AE4196-8FC4-4ED1-B0C4-588DEA137F80}">
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetData>
+    <row r="1" spans="1:18" ht="124" customHeight="1">
+      <c r="A1" s="45"/>
+      <c r="B1" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="48" t="s">
+        <v>217</v>
+      </c>
+      <c r="I1" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" s="48" t="s">
+        <v>218</v>
+      </c>
+      <c r="L1" s="43" t="s">
+        <v>219</v>
+      </c>
+      <c r="M1" s="43" t="s">
+        <v>219</v>
+      </c>
+      <c r="N1" s="48" t="s">
+        <v>222</v>
+      </c>
+      <c r="O1" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="P1" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q1" s="48" t="s">
+        <v>224</v>
+      </c>
+      <c r="R1" s="48" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="46.5">
+      <c r="A2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="M2" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="N2" s="49"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="R1:R2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:Q107"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
@@ -3940,7 +4159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:X9"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
@@ -3990,7 +4209,7 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4" t="s">
-        <v>144</v>
+        <v>215</v>
       </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -4209,7 +4428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B4:O4"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
@@ -4263,7 +4482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A3:I6"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
@@ -4324,7 +4543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A2:AD6"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
@@ -4483,7 +4702,7 @@
       </c>
       <c r="N4" s="15">
         <f ca="1">DATE(YEAR(TODAY()), MONTH(TODAY()+M4), DAY(TODAY()))</f>
-        <v>46068</v>
+        <v>46136</v>
       </c>
       <c r="O4" s="14"/>
       <c r="P4" s="14"/>
@@ -4524,14 +4743,14 @@
       <c r="K5" s="14"/>
       <c r="L5" s="15">
         <f ca="1">TODAY()</f>
-        <v>46037</v>
+        <v>46105</v>
       </c>
       <c r="M5" s="14">
         <v>21</v>
       </c>
       <c r="N5" s="15">
         <f ca="1">DATE(YEAR(L5),MONTH(L5)+M5,DAY(L5))</f>
-        <v>46675</v>
+        <v>46745</v>
       </c>
       <c r="O5" s="14"/>
       <c r="P5" s="14"/>

</xml_diff>